<commit_message>
Update main paper analysis outputs
</commit_message>
<xml_diff>
--- a/20251229_new_progress/Code/paper_data_newdata/main_paper_results/03_interpersonal_incremental_modeling/outputs/interpersonal_incremental_model_performance.xlsx
+++ b/20251229_new_progress/Code/paper_data_newdata/main_paper_results/03_interpersonal_incremental_modeling/outputs/interpersonal_incremental_model_performance.xlsx
@@ -449,7 +449,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -994,7 +994,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1023,37 +1023,37 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>0.743</v>
+        <v>0.74</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.761</v>
+        <v>0.756</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.766</v>
+        <v>0.768</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.764</v>
+        <v>0.762</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>0.741</v>
+        <v>0.738</v>
       </c>
       <c r="Q5" s="3" t="n">
         <v>0.736</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>0.734</v>
+        <v>0.735</v>
       </c>
       <c r="T5" s="3" t="n">
         <v>0.013</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>0.756</v>
+        <v>0.757</v>
       </c>
       <c r="V5" s="3" t="n">
-        <v>0.014</v>
+        <v>0.015</v>
       </c>
       <c r="W5" s="3" t="n">
         <v>0.8110000000000001</v>
@@ -1065,25 +1065,25 @@
         <v>0.757</v>
       </c>
       <c r="Z5" s="3" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="AA5" s="3" t="n">
-        <v>0.756</v>
+        <v>0.757</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>0.022</v>
+        <v>0.025</v>
       </c>
       <c r="AC5" s="3" t="n">
-        <v>0.756</v>
+        <v>0.757</v>
       </c>
       <c r="AD5" s="3" t="n">
-        <v>0.022</v>
+        <v>0.025</v>
       </c>
       <c r="AE5" s="3" t="n">
-        <v>0.713</v>
+        <v>0.712</v>
       </c>
       <c r="AF5" s="3" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="6">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1129,73 +1129,73 @@
         <v>42</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.630957</v>
+        <v>0.1</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0.8179999999999999</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.74</v>
+        <v>0.737</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.757</v>
+        <v>0.752</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.766</v>
+        <v>0.768</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.762</v>
+        <v>0.76</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.738</v>
+        <v>0.735</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.736</v>
+        <v>0.734</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.013</v>
+        <v>0.019</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>0.734</v>
+        <v>0.733</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>0.013</v>
+        <v>0.018</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>0.013</v>
+        <v>0.019</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="X6" s="3" t="n">
         <v>0.015</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>0.011</v>
+        <v>0.015</v>
       </c>
       <c r="AA6" s="3" t="n">
-        <v>0.756</v>
+        <v>0.754</v>
       </c>
       <c r="AB6" s="3" t="n">
-        <v>0.019</v>
+        <v>0.026</v>
       </c>
       <c r="AC6" s="3" t="n">
-        <v>0.756</v>
+        <v>0.754</v>
       </c>
       <c r="AD6" s="3" t="n">
-        <v>0.019</v>
+        <v>0.026</v>
       </c>
       <c r="AE6" s="3" t="n">
-        <v>0.712</v>
+        <v>0.711</v>
       </c>
       <c r="AF6" s="3" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="7">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1241,73 +1241,73 @@
         <v>42</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.039811</v>
+        <v>0.025119</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>0.8179999999999999</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>0.745</v>
+        <v>0.739</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.762</v>
+        <v>0.755</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.769</v>
+        <v>0.766</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.765</v>
+        <v>0.761</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0.743</v>
+        <v>0.736</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>0.736</v>
+        <v>0.734</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>0.013</v>
+        <v>0.016</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>0.735</v>
+        <v>0.732</v>
       </c>
       <c r="T7" s="3" t="n">
-        <v>0.012</v>
+        <v>0.015</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>0.757</v>
+        <v>0.754</v>
       </c>
       <c r="V7" s="3" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="W7" s="3" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="X7" s="3" t="n">
         <v>0.015</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>0.757</v>
+        <v>0.754</v>
       </c>
       <c r="Z7" s="3" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="AA7" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="AB7" s="3" t="n">
-        <v>0.021</v>
+        <v>0.025</v>
       </c>
       <c r="AC7" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="AD7" s="3" t="n">
-        <v>0.021</v>
+        <v>0.025</v>
       </c>
       <c r="AE7" s="3" t="n">
-        <v>0.713</v>
+        <v>0.709</v>
       </c>
       <c r="AF7" s="3" t="n">
-        <v>0.014</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="8">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1688,70 +1688,70 @@
       </c>
       <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="n">
-        <v>0.716</v>
+        <v>0.715</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0.653</v>
+        <v>0.655</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.668</v>
+        <v>0.67</v>
       </c>
       <c r="N11" s="3" t="n">
         <v>0.679</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.673</v>
+        <v>0.674</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.652</v>
+        <v>0.653</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0.647</v>
+        <v>0.649</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>0.646</v>
+        <v>0.648</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>0.666</v>
+        <v>0.668</v>
       </c>
       <c r="V11" s="3" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
       <c r="W11" s="3" t="n">
         <v>0.704</v>
       </c>
       <c r="X11" s="3" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>0.665</v>
+      </c>
+      <c r="Z11" s="3" t="n">
         <v>0.012</v>
       </c>
-      <c r="Y11" s="3" t="n">
-        <v>0.663</v>
-      </c>
-      <c r="Z11" s="3" t="n">
-        <v>0.015</v>
-      </c>
       <c r="AA11" s="3" t="n">
-        <v>0.669</v>
+        <v>0.671</v>
       </c>
       <c r="AB11" s="3" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="AC11" s="3" t="n">
-        <v>0.669</v>
+        <v>0.671</v>
       </c>
       <c r="AD11" s="3" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="AE11" s="3" t="n">
-        <v>0.623</v>
+        <v>0.624</v>
       </c>
       <c r="AF11" s="3" t="n">
-        <v>0.018</v>
+        <v>0.014</v>
       </c>
     </row>
     <row r="12">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1800,43 +1800,43 @@
         <v>0.063096</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.718</v>
+        <v>0.717</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.658</v>
+        <v>0.653</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.674</v>
+        <v>0.669</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.676</v>
+        <v>0.672</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.675</v>
+        <v>0.67</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.657</v>
+        <v>0.651</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.647</v>
+        <v>0.648</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.645</v>
+        <v>0.646</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="U12" s="3" t="n">
         <v>0.668</v>
       </c>
       <c r="V12" s="3" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="W12" s="3" t="n">
-        <v>0.705</v>
+        <v>0.704</v>
       </c>
       <c r="X12" s="3" t="n">
         <v>0.011</v>
@@ -1848,16 +1848,16 @@
         <v>0.013</v>
       </c>
       <c r="AA12" s="3" t="n">
-        <v>0.674</v>
+        <v>0.675</v>
       </c>
       <c r="AB12" s="3" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="AC12" s="3" t="n">
-        <v>0.674</v>
+        <v>0.675</v>
       </c>
       <c r="AD12" s="3" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="AE12" s="3" t="n">
         <v>0.617</v>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1912,70 +1912,70 @@
         <v>0.00631</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0.717</v>
+        <v>0.716</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0.659</v>
+        <v>0.653</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.672</v>
+        <v>0.668</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.678</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.679</v>
+        <v>0.673</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>0.657</v>
+        <v>0.652</v>
       </c>
       <c r="Q13" s="3" t="n">
         <v>0.648</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="S13" s="3" t="n">
         <v>0.646</v>
       </c>
       <c r="T13" s="3" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="U13" s="3" t="n">
         <v>0.669</v>
       </c>
       <c r="V13" s="3" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="W13" s="3" t="n">
         <v>0.705</v>
       </c>
       <c r="X13" s="3" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="Y13" s="3" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="Z13" s="3" t="n">
         <v>0.012</v>
       </c>
-      <c r="Y13" s="3" t="n">
-        <v>0.662</v>
-      </c>
-      <c r="Z13" s="3" t="n">
-        <v>0.015</v>
-      </c>
       <c r="AA13" s="3" t="n">
-        <v>0.676</v>
+        <v>0.678</v>
       </c>
       <c r="AB13" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AC13" s="3" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="AD13" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AE13" s="3" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="AF13" s="3" t="n">
         <v>0.016</v>
-      </c>
-      <c r="AC13" s="3" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="AD13" s="3" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="AE13" s="3" t="n">
-        <v>0.617</v>
-      </c>
-      <c r="AF13" s="3" t="n">
-        <v>0.018</v>
       </c>
     </row>
   </sheetData>
@@ -2257,55 +2257,55 @@
         <v>0.8110000000000001</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.001000000000000001</v>
+        <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>0.732</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.736</v>
+        <v>0.734</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.002000000000000002</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0.73</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.734</v>
+        <v>0.733</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.003000000000000003</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>0.751</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>0.005000000000000004</v>
+        <v>0.004000000000000004</v>
       </c>
       <c r="Q2" s="3" t="n">
         <v>0.757</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.756</v>
+        <v>0.754</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>-0.001000000000000001</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="T2" s="3" t="n">
         <v>0.754</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="V2" s="3" t="n">
-        <v>0.002000000000000002</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="W2" s="3" t="n">
         <v>0.8159999999999999</v>
@@ -2320,46 +2320,46 @@
         <v>0.74</v>
       </c>
       <c r="AA2" s="3" t="n">
-        <v>0.74</v>
+        <v>0.737</v>
       </c>
       <c r="AB2" s="3" t="n">
-        <v>0</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="AC2" s="3" t="n">
         <v>0.737</v>
       </c>
       <c r="AD2" s="3" t="n">
-        <v>0.738</v>
+        <v>0.735</v>
       </c>
       <c r="AE2" s="3" t="n">
-        <v>0.001000000000000001</v>
+        <v>-0.002000000000000002</v>
       </c>
       <c r="AF2" s="3" t="n">
         <v>0.754</v>
       </c>
       <c r="AG2" s="3" t="n">
-        <v>0.757</v>
+        <v>0.752</v>
       </c>
       <c r="AH2" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>-0.002000000000000002</v>
       </c>
       <c r="AI2" s="3" t="n">
         <v>0.769</v>
       </c>
       <c r="AJ2" s="3" t="n">
-        <v>0.766</v>
+        <v>0.768</v>
       </c>
       <c r="AK2" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="AL2" s="3" t="n">
         <v>0.762</v>
       </c>
       <c r="AM2" s="3" t="n">
-        <v>0.762</v>
+        <v>0.76</v>
       </c>
       <c r="AN2" s="3" t="n">
-        <v>0</v>
+        <v>-0.002000000000000002</v>
       </c>
     </row>
     <row r="3">
@@ -2401,10 +2401,10 @@
         <v>0.731</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>0.734</v>
+        <v>0.735</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>0.004000000000000004</v>
       </c>
       <c r="N3" s="3" t="n">
         <v>0.752</v>
@@ -2419,19 +2419,19 @@
         <v>0.758</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>0.756</v>
+        <v>0.757</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>-0.002000000000000002</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="T3" s="3" t="n">
         <v>0.755</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>0.756</v>
+        <v>0.757</v>
       </c>
       <c r="V3" s="3" t="n">
-        <v>0.001000000000000001</v>
+        <v>0.002000000000000002</v>
       </c>
       <c r="W3" s="3" t="n">
         <v>0.8159999999999999</v>
@@ -2446,46 +2446,46 @@
         <v>0.74</v>
       </c>
       <c r="AA3" s="3" t="n">
-        <v>0.743</v>
+        <v>0.74</v>
       </c>
       <c r="AB3" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="3" t="n">
         <v>0.737</v>
       </c>
       <c r="AD3" s="3" t="n">
-        <v>0.741</v>
+        <v>0.738</v>
       </c>
       <c r="AE3" s="3" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="AF3" s="3" t="n">
         <v>0.754</v>
       </c>
       <c r="AG3" s="3" t="n">
-        <v>0.761</v>
+        <v>0.756</v>
       </c>
       <c r="AH3" s="3" t="n">
-        <v>0.007000000000000006</v>
+        <v>0.002000000000000002</v>
       </c>
       <c r="AI3" s="3" t="n">
         <v>0.769</v>
       </c>
       <c r="AJ3" s="3" t="n">
-        <v>0.766</v>
+        <v>0.768</v>
       </c>
       <c r="AK3" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="AL3" s="3" t="n">
         <v>0.762</v>
       </c>
       <c r="AM3" s="3" t="n">
-        <v>0.764</v>
+        <v>0.762</v>
       </c>
       <c r="AN3" s="3" t="n">
-        <v>0.002000000000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2509,55 +2509,55 @@
         <v>0.8110000000000001</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.001000000000000001</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>0.734</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.736</v>
+        <v>0.734</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.002000000000000002</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0.732</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.735</v>
+        <v>0.732</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>0</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>0.752</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.757</v>
+        <v>0.754</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.005000000000000004</v>
+        <v>0.002000000000000002</v>
       </c>
       <c r="Q4" s="3" t="n">
         <v>0.758</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.756</v>
+        <v>0.755</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>-0.002000000000000002</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="T4" s="3" t="n">
         <v>0.755</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>0.757</v>
+        <v>0.754</v>
       </c>
       <c r="V4" s="3" t="n">
-        <v>0.002000000000000002</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="W4" s="3" t="n">
         <v>0.8159999999999999</v>
@@ -2572,46 +2572,46 @@
         <v>0.739</v>
       </c>
       <c r="AA4" s="3" t="n">
-        <v>0.745</v>
+        <v>0.739</v>
       </c>
       <c r="AB4" s="3" t="n">
-        <v>0.006000000000000005</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="3" t="n">
         <v>0.736</v>
       </c>
       <c r="AD4" s="3" t="n">
-        <v>0.743</v>
+        <v>0.736</v>
       </c>
       <c r="AE4" s="3" t="n">
-        <v>0.007000000000000006</v>
+        <v>0</v>
       </c>
       <c r="AF4" s="3" t="n">
         <v>0.753</v>
       </c>
       <c r="AG4" s="3" t="n">
-        <v>0.762</v>
+        <v>0.755</v>
       </c>
       <c r="AH4" s="3" t="n">
-        <v>0.009000000000000008</v>
+        <v>0.002000000000000002</v>
       </c>
       <c r="AI4" s="3" t="n">
         <v>0.769</v>
       </c>
       <c r="AJ4" s="3" t="n">
-        <v>0.769</v>
+        <v>0.766</v>
       </c>
       <c r="AK4" s="3" t="n">
-        <v>0</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="AL4" s="3" t="n">
         <v>0.761</v>
       </c>
       <c r="AM4" s="3" t="n">
-        <v>0.765</v>
+        <v>0.761</v>
       </c>
       <c r="AN4" s="3" t="n">
-        <v>0.004000000000000004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2635,28 +2635,28 @@
         <v>0.707</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.705</v>
+        <v>0.704</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.002000000000000002</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>0.647</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.647</v>
+        <v>0.648</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>0.645</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>0.645</v>
+        <v>0.646</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>0.661</v>
@@ -2671,10 +2671,10 @@
         <v>0.674</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0.674</v>
+        <v>0.675</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>0</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="T5" s="3" t="n">
         <v>0.668</v>
@@ -2689,55 +2689,55 @@
         <v>0.718</v>
       </c>
       <c r="X5" s="3" t="n">
-        <v>0.718</v>
+        <v>0.717</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>0</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="Z5" s="3" t="n">
         <v>0.655</v>
       </c>
       <c r="AA5" s="3" t="n">
-        <v>0.658</v>
+        <v>0.653</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>-0.002000000000000002</v>
       </c>
       <c r="AC5" s="3" t="n">
         <v>0.654</v>
       </c>
       <c r="AD5" s="3" t="n">
-        <v>0.657</v>
+        <v>0.651</v>
       </c>
       <c r="AE5" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="AF5" s="3" t="n">
         <v>0.672</v>
       </c>
       <c r="AG5" s="3" t="n">
-        <v>0.674</v>
+        <v>0.669</v>
       </c>
       <c r="AH5" s="3" t="n">
-        <v>0.002000000000000002</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="AI5" s="3" t="n">
         <v>0.671</v>
       </c>
       <c r="AJ5" s="3" t="n">
-        <v>0.676</v>
+        <v>0.672</v>
       </c>
       <c r="AK5" s="3" t="n">
-        <v>0.005000000000000004</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="AL5" s="3" t="n">
         <v>0.671</v>
       </c>
       <c r="AM5" s="3" t="n">
-        <v>0.675</v>
+        <v>0.67</v>
       </c>
       <c r="AN5" s="3" t="n">
-        <v>0.004000000000000004</v>
+        <v>-0.001000000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2770,82 +2770,82 @@
         <v>0.65</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.647</v>
+        <v>0.649</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0.649</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.646</v>
+        <v>0.648</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>0.666</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.663</v>
+        <v>0.665</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="Q6" s="3" t="n">
         <v>0.673</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.669</v>
+        <v>0.671</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>-0.004000000000000004</v>
+        <v>-0.002000000000000002</v>
       </c>
       <c r="T6" s="3" t="n">
         <v>0.669</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>0.666</v>
+        <v>0.668</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="W6" s="3" t="n">
         <v>0.717</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>0.716</v>
+        <v>0.715</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>-0.001000000000000001</v>
+        <v>-0.002000000000000002</v>
       </c>
       <c r="Z6" s="3" t="n">
         <v>0.656</v>
       </c>
       <c r="AA6" s="3" t="n">
-        <v>0.653</v>
+        <v>0.655</v>
       </c>
       <c r="AB6" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="AC6" s="3" t="n">
         <v>0.654</v>
       </c>
       <c r="AD6" s="3" t="n">
-        <v>0.652</v>
+        <v>0.653</v>
       </c>
       <c r="AE6" s="3" t="n">
-        <v>-0.002000000000000002</v>
+        <v>-0.001000000000000001</v>
       </c>
       <c r="AF6" s="3" t="n">
         <v>0.669</v>
       </c>
       <c r="AG6" s="3" t="n">
-        <v>0.668</v>
+        <v>0.67</v>
       </c>
       <c r="AH6" s="3" t="n">
-        <v>-0.001000000000000001</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="AI6" s="3" t="n">
         <v>0.6820000000000001</v>
@@ -2860,10 +2860,10 @@
         <v>0.676</v>
       </c>
       <c r="AM6" s="3" t="n">
-        <v>0.673</v>
+        <v>0.674</v>
       </c>
       <c r="AN6" s="3" t="n">
-        <v>-0.003000000000000003</v>
+        <v>-0.002000000000000002</v>
       </c>
     </row>
     <row r="7">
@@ -2914,19 +2914,19 @@
         <v>0.664</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.662</v>
+        <v>0.661</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>-0.002000000000000002</v>
+        <v>-0.003000000000000003</v>
       </c>
       <c r="Q7" s="3" t="n">
         <v>0.678</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>0.676</v>
+        <v>0.678</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>-0.002000000000000002</v>
+        <v>0</v>
       </c>
       <c r="T7" s="3" t="n">
         <v>0.671</v>
@@ -2941,55 +2941,55 @@
         <v>0.718</v>
       </c>
       <c r="X7" s="3" t="n">
-        <v>0.717</v>
+        <v>0.716</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>-0.001000000000000001</v>
+        <v>-0.002000000000000002</v>
       </c>
       <c r="Z7" s="3" t="n">
         <v>0.659</v>
       </c>
       <c r="AA7" s="3" t="n">
-        <v>0.659</v>
+        <v>0.653</v>
       </c>
       <c r="AB7" s="3" t="n">
-        <v>0</v>
+        <v>-0.006000000000000005</v>
       </c>
       <c r="AC7" s="3" t="n">
         <v>0.657</v>
       </c>
       <c r="AD7" s="3" t="n">
-        <v>0.657</v>
+        <v>0.652</v>
       </c>
       <c r="AE7" s="3" t="n">
-        <v>0</v>
+        <v>-0.005000000000000004</v>
       </c>
       <c r="AF7" s="3" t="n">
         <v>0.673</v>
       </c>
       <c r="AG7" s="3" t="n">
-        <v>0.672</v>
+        <v>0.668</v>
       </c>
       <c r="AH7" s="3" t="n">
-        <v>-0.001000000000000001</v>
+        <v>-0.005000000000000004</v>
       </c>
       <c r="AI7" s="3" t="n">
         <v>0.6830000000000001</v>
       </c>
       <c r="AJ7" s="3" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.678</v>
       </c>
       <c r="AK7" s="3" t="n">
-        <v>0.003000000000000003</v>
+        <v>-0.005000000000000004</v>
       </c>
       <c r="AL7" s="3" t="n">
         <v>0.678</v>
       </c>
       <c r="AM7" s="3" t="n">
-        <v>0.679</v>
+        <v>0.673</v>
       </c>
       <c r="AN7" s="3" t="n">
-        <v>0.001000000000000001</v>
+        <v>-0.005000000000000004</v>
       </c>
     </row>
   </sheetData>
@@ -3012,7 +3012,7 @@
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
     <col width="41" customWidth="1" min="6" max="6"/>
-    <col width="57" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="39" customWidth="1" min="9" max="9"/>
   </cols>
@@ -3079,13 +3079,13 @@
         <v>12</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>9.801653519417476</v>
+        <v>5.193099610461881</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>2.188258495145631</v>
+        <v>1.627156371730662</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -3093,10 +3093,10 @@
         </is>
       </c>
       <c r="H2" s="3" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -3114,13 +3114,13 @@
         <v>12</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>11.46047391296441</v>
+        <v>10.54754406320791</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2.245903726199786</v>
+        <v>1.96880122290366</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -3147,13 +3147,13 @@
         <v>12</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>11.02646196574603</v>
+        <v>9.906865407438699</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2.162089183767937</v>
+        <v>1.834530203367329</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="H4" s="3" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
     </row>
@@ -3180,21 +3180,21 @@
         <v>12</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3.171718089698731</v>
+        <v>3.952818296416352</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2.190212205207434</v>
+        <v>1.629749684855033</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Reciprocal Friendship Ties, Respondent-Class-Normalized</t>
+          <t>Reciprocal Friendship Ties, Observed Count</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>4</v>
@@ -3218,18 +3218,18 @@
         <v>2</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>13.99327731092437</v>
+        <v>13.72118921472682</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3.811764705882353</v>
+        <v>3.408362298788513</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Reciprocal Friendship Ties, Respondent-Class-Normalized</t>
+          <t>Reciprocal Friendship Ties, Observed Count</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I6" s="3" t="inlineStr"/>
     </row>
@@ -3251,18 +3251,18 @@
         <v>1</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>10.46618831923678</v>
+        <v>10.56721679218074</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2.729787148755361</v>
+        <v>2.519628264701169</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Reciprocal Friendship Ties, Respondent-Class-Normalized</t>
+          <t>Reciprocal Friendship Ties, Observed Count</t>
         </is>
       </c>
       <c r="H7" s="3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I7" s="3" t="inlineStr"/>
     </row>
@@ -3291,7 +3291,7 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="49" customWidth="1" min="12" max="12"/>
     <col width="70" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -3646,12 +3646,12 @@
       </c>
       <c r="Z3" s="3" t="inlineStr">
         <is>
-          <t>respondent_class_normalized</t>
+          <t>observed_count</t>
         </is>
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>ip_online_total_rate_class;ip_offline_total_rate_class;ip_out_friend_total_rate_class;ip_in_friend_total_rate_class;ip_out_enemy_total_rate_class;ip_in_enemy_total_rate_class;ip_reciprocal_friend_count_rate_class;ip_reciprocal_enemy_count_rate_class;ip_sent_like_ratio;ip_received_like_ratio;ip_sent_net_rate_class;ip_received_net_rate_class</t>
+          <t>ip_online_total;ip_offline_total;ip_out_friend_total;ip_in_friend_total;ip_out_enemy_total;ip_in_enemy_total;ip_reciprocal_friend_count;ip_reciprocal_enemy_count;ip_sent_like_ratio;ip_received_like_ratio;ip_sent_net;ip_received_net</t>
         </is>
       </c>
       <c r="AB3" s="3" t="inlineStr"/>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Decomposed + 12 interpersonal features</t>
+          <t>Decomposed + 12 observed interpersonal features</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -3850,12 +3850,12 @@
       </c>
       <c r="Z5" s="3" t="inlineStr">
         <is>
-          <t>respondent_class_normalized</t>
+          <t>observed_count</t>
         </is>
       </c>
       <c r="AA5" s="3" t="inlineStr">
         <is>
-          <t>ip_online_total_rate_class;ip_offline_total_rate_class;ip_out_friend_total_rate_class;ip_in_friend_total_rate_class;ip_out_enemy_total_rate_class;ip_in_enemy_total_rate_class;ip_reciprocal_friend_count_rate_class;ip_reciprocal_enemy_count_rate_class;ip_sent_like_ratio;ip_received_like_ratio;ip_sent_net_rate_class;ip_received_net_rate_class</t>
+          <t>ip_online_total;ip_offline_total;ip_out_friend_total;ip_in_friend_total;ip_out_enemy_total;ip_in_enemy_total;ip_reciprocal_friend_count;ip_reciprocal_enemy_count;ip_sent_like_ratio;ip_received_like_ratio;ip_sent_net;ip_received_net</t>
         </is>
       </c>
       <c r="AB5" s="3" t="inlineStr"/>

</xml_diff>